<commit_message>
fix: complete all 51 Meesho product URLs with ?ms=2&source=Meri+Shop store parameters
</commit_message>
<xml_diff>
--- a/spice-nest-hub/output/meesho_store_tracker.xlsx
+++ b/spice-nest-hub/output/meesho_store_tracker.xlsx
@@ -695,7 +695,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated at: 2026-10-31 16:02:28 | Target: Spice Nest Impex Private Limited</t>
+          <t>Generated at: 2026-10-31 16:17:05 | Target: Spice Nest Impex Private Limited</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="M2" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/fruity-delight-jam-pack-strawberry-pineapple-mixed-fruit-jars-combo/p/djcu1d</t>
+          <t>https://www.meesho.com/fruity-delight-jam-pack-strawberry-pineapple-mixed-fruit-jars-combo/p/djcu1d?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N2" s="13" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="M3" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-red-chilli-oil-450g-hot-spicy-chilli-garlic-crisp-for-momos-noodles-fried-rice-pizza-pasta-tadka-cooking/p/fix7tb</t>
+          <t>https://www.meesho.com/spice-nest-red-chilli-oil-450g-hot-spicy-chilli-garlic-crisp-for-momos-noodles-fried-rice-pizza-pasta-tadka-cooking/p/fix7tb?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N3" s="13" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-premium-mix-fruit-jam-370g-strawberry-jam-370g-combo-rich-natural-flavor-for-your-breakfast-and-snacks/p/aykhr0</t>
+          <t>https://www.meesho.com/spice-nest-premium-mix-fruit-jam-370g-strawberry-jam-370g-combo-rich-natural-flavor-for-your-breakfast-and-snacks/p/aykhr0?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N4" s="13" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mix-fruit-jam-pineapple-jam-370g-combo-pack-pure-homemade-spread-no-preservatives/p/ayrop3</t>
+          <t>https://www.meesho.com/spice-nest-mix-fruit-jam-pineapple-jam-370g-combo-pack-pure-homemade-spread-no-preservatives/p/ayrop3?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N5" s="13" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-strawberry-jam-370g-pineapple-jam-370g-twin-pack-perfect-for-daily-snacks-cakes-gifts/p/ayz2yo</t>
+          <t>https://www.meesho.com/spice-nest-strawberry-jam-370g-pineapple-jam-370g-twin-pack-perfect-for-daily-snacks-cakes-gifts/p/ayz2yo?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N6" s="13" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-370g-mix-fruit-pineapple-jam-pack-fresh-fruit-spread-combo/p/azu93e</t>
+          <t>https://www.meesho.com/spice-nest-370g-mix-fruit-pineapple-jam-pack-fresh-fruit-spread-combo/p/azu93e?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N7" s="13" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/sweet-lemon-pickle-200-g-each-pack-of-3/p/hofy3n</t>
+          <t>https://www.meesho.com/sweet-lemon-pickle-200-g-each-pack-of-3/p/hofy3n?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mix-fruit-jam-370g-apricot-jam-370g-combo-pack-pure-spread-delight/p/aztlwe</t>
+          <t>https://www.meesho.com/spice-nest-mix-fruit-jam-370g-apricot-jam-370g-combo-pack-pure-spread-delight/p/aztlwe?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N9" s="13" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="M10" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-370g-mix-fruit-strawberry-jam-duo-classic-fruit-spread-deal/p/azu9z6</t>
+          <t>https://www.meesho.com/spice-nest-370g-mix-fruit-strawberry-jam-duo-classic-fruit-spread-deal/p/azu9z6?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N10" s="13" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-strawberry-jam-370gm-raspberry-jam-370gm-combo-a-perfect-pair-of-sweet-and-tangy-flavors-for-spreads-desserts-and-more/p/b0i9ej</t>
+          <t>https://www.meesho.com/spice-nest-strawberry-jam-370gm-raspberry-jam-370gm-combo-a-perfect-pair-of-sweet-and-tangy-flavors-for-spreads-desserts-and-more/p/b0i9ej?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N11" s="13" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="M12" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-strawberry-jam-370gm-pineapple-jam-370gm-combo-perfect-blend-of-sweet-tangy-flavors-for-spreads-desserts-and-snacks/p/b0i8lu</t>
+          <t>https://www.meesho.com/spice-nest-strawberry-jam-370gm-pineapple-jam-370gm-combo-perfect-blend-of-sweet-tangy-flavors-for-spreads-desserts-and-snacks/p/b0i8lu?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N12" s="13" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mix-fruit-jam-apricot-jam-370g-combo-pack-pure-homemade-spread-no-preservatives/p/aymssf</t>
+          <t>https://www.meesho.com/spice-nest-mix-fruit-jam-apricot-jam-370g-combo-pack-pure-homemade-spread-no-preservatives/p/aymssf?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N13" s="13" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/mix-fruit-jam-1kg/p/9220r3</t>
+          <t>https://www.meesho.com/mix-fruit-jam-1kg/p/9220r3?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N14" s="13" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="M15" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/garlic-pickle-500g-pack-of-2-savoury-spiced-and-tangy-indian-style-pickle-combo/p/h36cl9</t>
+          <t>https://www.meesho.com/garlic-pickle-500g-pack-of-2-savoury-spiced-and-tangy-indian-style-pickle-combo/p/h36cl9?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N15" s="13" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="M16" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/red-chilli-pickle-500g-pack-of-2-authentic-spiced-and-tangy-red-chilli-pickle-combo/p/h36clx</t>
+          <t>https://www.meesho.com/red-chilli-pickle-500g-pack-of-2-authentic-spiced-and-tangy-red-chilli-pickle-combo/p/h36clx?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N16" s="13" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/green-chilli-pickle-500g-pack-of-2-authentic-spiced-and-tangy-green-chilli-pickle-combo/p/h36clf</t>
+          <t>https://www.meesho.com/green-chilli-pickle-500g-pack-of-2-authentic-spiced-and-tangy-green-chilli-pickle-combo/p/h36clf?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N17" s="13" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="M18" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/mixed-pickle-500g-pack-of-2-assorted-vegetable-spiced-and-homemade-style-pickle-combo/p/h36clc</t>
+          <t>https://www.meesho.com/mixed-pickle-500g-pack-of-2-assorted-vegetable-spiced-and-homemade-style-pickle-combo/p/h36clc?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N18" s="13" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="M19" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-strawberry-jam-370gm/p/aen2qe</t>
+          <t>https://www.meesho.com/spice-nest-strawberry-jam-370gm/p/aen2qe?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N19" s="13" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mixed-fruit-jam-370gm-made-with-real-fruits-no-artificial-flavors/p/abk64v</t>
+          <t>https://www.meesho.com/spice-nest-mixed-fruit-jam-370gm-made-with-real-fruits-no-artificial-flavors/p/abk64v?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N20" s="13" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="M21" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mixed-pickle-garlic-pickle-combo-500g-each-pack-of-2-indian-achar-for-roti-paratha-rice-meals/p/h0jvhs</t>
+          <t>https://www.meesho.com/spice-nest-mixed-pickle-garlic-pickle-combo-500g-each-pack-of-2-indian-achar-for-roti-paratha-rice-meals/p/h0jvhs?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N21" s="13" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="M22" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-garlic-pickle-1kg-premium-homemade-style-garlic-achar/p/h36cl2</t>
+          <t>https://www.meesho.com/spice-nest-garlic-pickle-1kg-premium-homemade-style-garlic-achar/p/h36cl2?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N22" s="13" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-ginger-garlic-paste-premium-fresh-natural-thick-aromatic-ready-to-use-cooking-essential-for-curries-marinades-soups-stir-fries-preservative-free-pack-of-2-ginger-garlic-paste-500gm/p/a1e9p0</t>
+          <t>https://www.meesho.com/spice-nest-ginger-garlic-paste-premium-fresh-natural-thick-aromatic-ready-to-use-cooking-essential-for-curries-marinades-soups-stir-fries-preservative-free-pack-of-2-ginger-garlic-paste-500gm/p/a1e9p0?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N23" s="13" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="M24" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mix-pickle-1kg-premium-mixed-vegetable-pickle/p/h36cko</t>
+          <t>https://www.meesho.com/spice-nest-mix-pickle-1kg-premium-mixed-vegetable-pickle/p/h36cko?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N24" s="13" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="M25" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/garlic-pickle-200-g-each-pack-of-3/p/hofsqs</t>
+          <t>https://www.meesho.com/garlic-pickle-200-g-each-pack-of-3/p/hofsqs?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N25" s="13" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="M26" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-garlic-paste-ready-to-use-lahsun-paste-naturally-processed-fresh-homemade-ingredients-no-added-flavor-or-preservatives-premium-quality-thick-aromatic-garlic-paste-for-cooking-1000gm-pack-of-1/p/9zbyw5</t>
+          <t>https://www.meesho.com/spice-nest-garlic-paste-ready-to-use-lahsun-paste-naturally-processed-fresh-homemade-ingredients-no-added-flavor-or-preservatives-premium-quality-thick-aromatic-garlic-paste-for-cooking-1000gm-pack-of-1/p/9zbyw5?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N26" s="13" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="M27" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/aromatic-ginger-garlic-paste-spice-nest-750gm-jar/p/axx39n</t>
+          <t>https://www.meesho.com/aromatic-ginger-garlic-paste-spice-nest-750gm-jar/p/axx39n?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N27" s="13" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="M28" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/red-chilli-green-chilli-soya-sauce-220gm-each-combo-sauce/p/8uplk7</t>
+          <t>https://www.meesho.com/red-chilli-green-chilli-soya-sauce-220gm-each-combo-sauce/p/8uplk7?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N28" s="13" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="M29" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mixed-fruit-jam-370gm-made-with-real-fruits-delicious-healthy-spread/p/abk09h</t>
+          <t>https://www.meesho.com/spice-nest-mixed-fruit-jam-370gm-made-with-real-fruits-delicious-healthy-spread/p/abk09h?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N29" s="13" t="inlineStr">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="M30" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-green-chilli-oil-120g-spicy-green-mirchi-flavour-oil-for-momos-noodles-fried-rice-pasta-rolls-snacks-daily-cooking/p/fggmdx</t>
+          <t>https://www.meesho.com/spice-nest-green-chilli-oil-120g-spicy-green-mirchi-flavour-oil-for-momos-noodles-fried-rice-pasta-rolls-snacks-daily-cooking/p/fggmdx?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N30" s="13" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="M31" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-red-chilli-oil-120g-hot-spicy-chilli-garlic-crisp-for-momos-noodles-fried-rice-pizza-pasta-tadka-cooking/p/fgfvjf</t>
+          <t>https://www.meesho.com/spice-nest-red-chilli-oil-120g-hot-spicy-chilli-garlic-crisp-for-momos-noodles-fried-rice-pizza-pasta-tadka-cooking/p/fgfvjf?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N31" s="13" t="inlineStr">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/mixed-fruit-jam-by-spice-nest/p/828zt5</t>
+          <t>https://www.meesho.com/mixed-fruit-jam-by-spice-nest/p/828zt5?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N32" s="13" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="M33" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mixed-pickle-combo-pack-500g-200g-traditional-indian-achar-spicy-tangy-pickle-for-roti-paratha-rice-and-dal-total-700g/p/h0jvhu</t>
+          <t>https://www.meesho.com/spice-nest-mixed-pickle-combo-pack-500g-200g-traditional-indian-achar-spicy-tangy-pickle-for-roti-paratha-rice-and-dal-total-700g/p/h0jvhu?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N33" s="13" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="M34" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/apricot-jam-370gm/p/92e7on</t>
+          <t>https://www.meesho.com/apricot-jam-370gm/p/92e7on?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N34" s="13" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="M35" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/premium-quality-ginger-garlic-paste-750gm-by-spice-nest/p/axxpmt</t>
+          <t>https://www.meesho.com/premium-quality-ginger-garlic-paste-750gm-by-spice-nest/p/axxpmt?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N35" s="13" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="M36" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-ginger-garlic-paste-750g-pure-adrak-lehsun-paste-no-preservatives-fresh-ginger-garlic-for-curries-biryani-indian-cooking-ready-to-use-jar/p/axi3yp</t>
+          <t>https://www.meesho.com/spice-nest-ginger-garlic-paste-750g-pure-adrak-lehsun-paste-no-preservatives-fresh-ginger-garlic-for-curries-biryani-indian-cooking-ready-to-use-jar/p/axi3yp?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N36" s="13" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="M37" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mixed-fruit-jam-370-gm-pack-of-1/p/abgtow</t>
+          <t>https://www.meesho.com/spice-nest-mixed-fruit-jam-370-gm-pack-of-1/p/abgtow?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N37" s="13" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="M38" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/ready-to-eat-paneer-tikka-masala-gravy-base-spicy-smoky-creamy-indian-curry-heat-and-eat-curry-authentic-north-indian-ready-meal-no-preservatives-300g-pack-pack-of-1-paneer-tika-masala-300-gm/p/ap5y65</t>
+          <t>https://www.meesho.com/ready-to-eat-paneer-tikka-masala-gravy-base-spicy-smoky-creamy-indian-curry-heat-and-eat-curry-authentic-north-indian-ready-meal-no-preservatives-300g-pack-pack-of-1-paneer-tika-masala-300-gm/p/ap5y65?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N38" s="13" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="M39" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-jhal-muri-sauce-230g-spicy-tangy-bengali-street-style-flavor/p/fsqsgb</t>
+          <t>https://www.meesho.com/spice-nest-jhal-muri-sauce-230g-spicy-tangy-bengali-street-style-flavor/p/fsqsgb?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N39" s="13" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="M40" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/garlic-pickle-200-g-each-pack-of-2/p/hofryh</t>
+          <t>https://www.meesho.com/garlic-pickle-200-g-each-pack-of-2/p/hofryh?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N40" s="13" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="M41" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-red-chilli-pickle-spicy-tangy-authentic-indian-achar-made-with-sun-dried-red-chilies-and-traditional-spices-preservative-free-homemade-style-pickle-for-parathas-rice-curries-meals-pack-of-1-red-chilli-pickle-500gm/p/ailpze</t>
+          <t>https://www.meesho.com/spice-nest-red-chilli-pickle-spicy-tangy-authentic-indian-achar-made-with-sun-dried-red-chilies-and-traditional-spices-preservative-free-homemade-style-pickle-for-parathas-rice-curries-meals-pack-of-1-red-chilli-pickle-500gm/p/ailpze?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N41" s="13" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="M42" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/premium-green-chilli-pickle-500gm/p/8fje2u</t>
+          <t>https://www.meesho.com/premium-green-chilli-pickle-500gm/p/8fje2u?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N42" s="13" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="M43" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-schezwan-sauce-250ml/p/cunvk5</t>
+          <t>https://www.meesho.com/spice-nest-schezwan-sauce-250ml/p/cunvk5?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N43" s="13" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="M44" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-garlic-pickle-500g-mixed-pickle-200g-combo-indian-achar-pack-of-2-total-700g/p/h0jvht</t>
+          <t>https://www.meesho.com/spice-nest-garlic-pickle-500g-mixed-pickle-200g-combo-indian-achar-pack-of-2-total-700g/p/h0jvht?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N44" s="13" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="M45" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/pineapple-jam-740gm-370370gm/p/86o55m</t>
+          <t>https://www.meesho.com/pineapple-jam-740gm-370370gm/p/86o55m?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N45" s="13" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="M46" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-classic-strawberry-jam-370gm-made-from-fresh-strawberries/p/aeuvav</t>
+          <t>https://www.meesho.com/spice-nest-classic-strawberry-jam-370gm-made-from-fresh-strawberries/p/aeuvav?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N46" s="13" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="M47" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-hot-spicy-chilli-oil-120gm-perfect-for-momos-noodles-fried-rice/p/ewkkta</t>
+          <t>https://www.meesho.com/spice-nest-hot-spicy-chilli-oil-120gm-perfect-for-momos-noodles-fried-rice/p/ewkkta?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N47" s="13" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="M48" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/pineapple-jam-370gm-jar/p/85k4dq</t>
+          <t>https://www.meesho.com/pineapple-jam-370gm-jar/p/85k4dq?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N48" s="13" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="M49" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spicy-tangy-garlic-pickle-200gm/p/86cube</t>
+          <t>https://www.meesho.com/spicy-tangy-garlic-pickle-200gm/p/86cube?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N49" s="13" t="inlineStr">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="M50" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-green-chilli-oil-120gm-spicy-flavoring-oil-for-cooking-tadka/p/ewjvdj</t>
+          <t>https://www.meesho.com/spice-nest-green-chilli-oil-120gm-spicy-flavoring-oil-for-cooking-tadka/p/ewjvdj?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N50" s="13" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="M51" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/dark-soya-sauce-220gm-bottle/p/85k06f</t>
+          <t>https://www.meesho.com/dark-soya-sauce-220gm-bottle/p/85k06f?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N51" s="13" t="inlineStr">
@@ -3922,7 +3922,7 @@
       </c>
       <c r="M52" s="13" t="inlineStr">
         <is>
-          <t>https://www.meesho.com/spice-nest-mixed-pickle-200gm-pack-of-1/p/81ocey</t>
+          <t>https://www.meesho.com/spice-nest-mixed-pickle-200gm-pack-of-1/p/81ocey?ms=2&amp;source=Meri+Shop</t>
         </is>
       </c>
       <c r="N52" s="13" t="inlineStr">

</xml_diff>